<commit_message>
Step 6: approval_ui.py Panel dashboard working
</commit_message>
<xml_diff>
--- a/data/output/master_repo.xlsx
+++ b/data/output/master_repo.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\OneDrive\Documents\Learning\Project\AgentBuild\data\output\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28EC52F1-F3DE-4EA0-BED1-DF8F35FFC372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
   <si>
     <t>issue_id</t>
   </si>
@@ -82,6 +76,9 @@
     <t>SNW-004</t>
   </si>
   <si>
+    <t>SNW-008</t>
+  </si>
+  <si>
     <t>CSV</t>
   </si>
   <si>
@@ -97,6 +94,9 @@
     <t>Workflow approval email notifications not sending</t>
   </si>
   <si>
+    <t>Active workspace not loading dashboard widgets</t>
+  </si>
+  <si>
     <t>Restart AMS service and apply hotfix KB-1042</t>
   </si>
   <si>
@@ -109,6 +109,9 @@
     <t>Reconfigure SMTP settings in TC admin panel</t>
   </si>
   <si>
+    <t>Clear active workspace cache and redeploy widgets</t>
+  </si>
+  <si>
     <t>Application Error</t>
   </si>
   <si>
@@ -121,6 +124,9 @@
     <t>Workflow</t>
   </si>
   <si>
+    <t>UI</t>
+  </si>
+  <si>
     <t>P2</t>
   </si>
   <si>
@@ -136,9 +142,15 @@
     <t>Subrasethu</t>
   </si>
   <si>
+    <t>KANNAN</t>
+  </si>
+  <si>
     <t>2026-03-30 07:29:30</t>
   </si>
   <si>
+    <t>2026-04-08 08:19:31</t>
+  </si>
+  <si>
     <t>Validated</t>
   </si>
   <si>
@@ -154,10 +166,19 @@
     <t>SOP-TC-2025-089</t>
   </si>
   <si>
+    <t>SOP-AMS-2025-021</t>
+  </si>
+  <si>
     <t>Active</t>
   </si>
   <si>
     <t>Subrasethu (SUB001)</t>
+  </si>
+  <si>
+    <t>2026-04-08 08:19:12</t>
+  </si>
+  <si>
+    <t>2026-04-08 08:19:13</t>
   </si>
   <si>
     <t>Excel plugin v3.2 replaced by v4.0</t>
@@ -169,8 +190,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -233,21 +254,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -285,7 +298,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -319,7 +332,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -354,10 +366,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -530,25 +541,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="6.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="47.81640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="37.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.36328125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -598,186 +595,227 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I2" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J2" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="K2" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="L2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="P2">
         <v>0.75</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G3" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I3" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="K3" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="L3" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="M3" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="N3" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="O3" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="P3">
         <v>0.75</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="L4" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="M4" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="N4" t="s">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="O4" t="s">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="P4">
         <v>0.75</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H5" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="J5" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="K5" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="L5" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="P5">
         <v>0.71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" t="s">
+        <v>36</v>
+      </c>
+      <c r="F6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I6" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" t="s">
+        <v>45</v>
+      </c>
+      <c r="K6" t="s">
+        <v>50</v>
+      </c>
+      <c r="L6" t="s">
+        <v>51</v>
+      </c>
+      <c r="P6">
+        <v>0.6222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Step 7: main.py complete agent pipeline working
</commit_message>
<xml_diff>
--- a/data/output/master_repo.xlsx
+++ b/data/output/master_repo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="63">
   <si>
     <t>issue_id</t>
   </si>
@@ -79,6 +79,9 @@
     <t>SNW-008</t>
   </si>
   <si>
+    <t>SNW-011</t>
+  </si>
+  <si>
     <t>CSV</t>
   </si>
   <si>
@@ -97,6 +100,9 @@
     <t>Active workspace not loading dashboard widgets</t>
   </si>
   <si>
+    <t>test the issue availability</t>
+  </si>
+  <si>
     <t>Restart AMS service and apply hotfix KB-1042</t>
   </si>
   <si>
@@ -112,6 +118,9 @@
     <t>Clear active workspace cache and redeploy widgets</t>
   </si>
   <si>
+    <t>Just a demo trial</t>
+  </si>
+  <si>
     <t>Application Error</t>
   </si>
   <si>
@@ -127,6 +136,9 @@
     <t>UI</t>
   </si>
   <si>
+    <t>Data</t>
+  </si>
+  <si>
     <t>P2</t>
   </si>
   <si>
@@ -145,10 +157,16 @@
     <t>KANNAN</t>
   </si>
   <si>
+    <t>SUBRASETHU</t>
+  </si>
+  <si>
     <t>2026-03-30 07:29:30</t>
   </si>
   <si>
     <t>2026-04-08 08:19:31</t>
+  </si>
+  <si>
+    <t>2026-04-08 22:41:20</t>
   </si>
   <si>
     <t>Validated</t>
@@ -542,7 +560,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
@@ -600,37 +618,37 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K2" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="L2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="P2">
         <v>0.75</v>
@@ -641,46 +659,46 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H3" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="K3" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="L3" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="M3" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="N3" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="O3" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="P3">
         <v>0.75</v>
@@ -691,46 +709,46 @@
         <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I4" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K4" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="L4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="M4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="N4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="O4" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="P4">
         <v>0.75</v>
@@ -741,37 +759,37 @@
         <v>19</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F5" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I5" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="J5" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K5" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="L5" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="P5">
         <v>0.71</v>
@@ -782,40 +800,78 @@
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I6" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="J6" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="L6" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="P6">
         <v>0.6222</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+      <c r="I7" t="s">
+        <v>50</v>
+      </c>
+      <c r="J7" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" t="s">
+        <v>57</v>
+      </c>
+      <c r="P7">
+        <v>0.5011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>